<commit_message>
fixed fileio bug with reinforcement lines. fixed some input templates that were not compatible with version 6.
</commit_message>
<xml_diff>
--- a/inputs/slope/input_template_reinf6.xlsx
+++ b/inputs/slope/input_template_reinf6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10727"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/cursor_projects/xslope/inputs/slope/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D771216D-4B03-C948-8921-267E39D1FD42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F0B0FC9-A496-B94B-826B-2C736DD848BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32260" yWindow="2140" windowWidth="29340" windowHeight="17300" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="5840" yWindow="2980" windowWidth="29340" windowHeight="17300" activeTab="5" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="139">
   <si>
     <t>X</t>
   </si>
@@ -6366,16 +6366,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="G22:H22"/>
     <mergeCell ref="J22:K22"/>
     <mergeCell ref="M22:N22"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7230,16 +7230,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3">
-        <v>500</v>
+        <v>50</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>26</v>
       </c>
       <c r="E3" s="3">
-        <v>197</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -7255,18 +7255,10 @@
       <c r="A4" s="3">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
-        <v>100</v>
-      </c>
-      <c r="C4" s="3">
-        <v>500</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="3">
-        <v>182</v>
-      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>

</xml_diff>